<commit_message>
Unify design terminology and trim tools
</commit_message>
<xml_diff>
--- a/spec/Docs/01_Design/OrnamentDesignVersion/饰品列表.xlsx
+++ b/spec/Docs/01_Design/OrnamentDesignVersion/饰品列表.xlsx
@@ -220,12 +220,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>每条撞击链第一次命中物品：+2分。</t>
+          <t>每次撞击结算第一次命中物品：+2分。</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>根源之梦；棒球；机械链</t>
+          <t>根源之梦；棒球；机械传动</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -327,7 +327,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>高San物品；特殊物品</t>
+          <t>高梦值消耗物品；特殊物品</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -531,7 +531,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>机械链；长条物品</t>
+          <t>机械传动；长条物品</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>废弃物完成结算后：若其有污染，+其污染层数分。每个物品每条链限1次。</t>
+          <t>废弃物完成结算后：若其有污染，+其污染层数分。每个物品每次撞击结算限1次。</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1036,7 +1036,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>污染层数大于等于3的物品完成结算后：+5分。每个物品每条链限1次。</t>
+          <t>污染层数大于等于3的物品完成结算后：+5分。每个物品每次撞击结算限1次。</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>污染层数大于等于5的物品完成结算后：+污染层数x2分。每个物品每条链限1次。</t>
+          <t>污染层数大于等于5的物品完成结算后：+污染层数x2分。每个物品每次撞击结算限1次。</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1796,12 +1796,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>机械/撞击链</t>
+          <t>机械/撞击结算</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>撞击链命中大于等于3个物品时：链结束+8分。</t>
+          <t>本次撞击结算命中大于等于3个物品时：在本次撞击结算全部停止后+8分。</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>鼓励玩家做长链。</t>
+          <t>鼓励玩家做长路径。</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -1852,7 +1852,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>每条撞击链中，第一个被撞物品如果方向与撞击来源相同：+5分。</t>
+          <t>每次撞击结算中，第一个被撞物品如果方向与撞击来源相同：+5分。</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -1877,7 +1877,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>链长计数器</t>
+          <t>命中计数器</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1898,12 +1898,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>机械/撞击链</t>
+          <t>机械/撞击结算</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>链结束：+本次命中物品数量分。若命中大于等于6，额外+8分。</t>
+          <t>本次撞击结算全部停止后：+本次命中物品数分。若命中大于等于6，额外+8分。</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -1913,7 +1913,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>把链长直接转化为收益。</t>
+          <t>把命中数直接转化为收益。</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>每条撞击链第一次命中机械物品：+6分。</t>
+          <t>每次撞击结算第一次命中机械物品：+6分。</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2005,17 +2005,17 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>机械物品成功传导撞击或曲线传动命中机械物品时：+2分，每条链最多触发5次。</t>
+          <t>机械物品成功传导撞击或曲线传动命中机械物品时：+2分，每次撞击结算最多触发5次。</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>机械长链；链长计数器；顺转弯管</t>
+          <t>机械长路径；命中计数器；左传动弯管</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>奖励机械链持续传导。</t>
+          <t>奖励机械传动持续传导。</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -2056,17 +2056,17 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>每个局内关卡第一次撞击链停止时，若最后被撞物品是机械：从该物品反方向发起一次机械撞击！</t>
+          <t>每个局内关卡第一次满足以下条件时触发：一次撞击结算全部停止后，最后被撞物品是机械。效果：从该物品反方向发起一次机械撞击！</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>机械链；终端压力表</t>
+          <t>机械传动；终端压力表</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>给机械链提供一次补偿性延伸。</t>
+          <t>给机械传动提供一次补偿性延伸。</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -2107,12 +2107,12 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>每条链第一次命中机械物品时：该物品本次触发双向传动！每条链限1次。</t>
+          <t>每次撞击结算第一次命中机械物品时：该物品本次触发双向传动！每次撞击结算限1次。</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>双轴转轮；曲线传动；长链</t>
+          <t>双轴转轮；曲线传动；长路径</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -2163,7 +2163,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>根源之梦；棒球；机械链</t>
+          <t>根源之梦；棒球；机械传动</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -2209,12 +2209,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>链结束：若本次链机械命中数大于等于8，+25分；若大于等于12，改为+45分。</t>
+          <t>本次撞击结算全部停止后：若本次命中机械物品数大于等于8，+25分；若大于等于12，改为+45分。</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>机械高阶长链；中央引擎；计数轮</t>
+          <t>机械高阶长路径；中央引擎；计数轮</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>每条撞击链命中3种或以上不同标签的物品：+15分。</t>
+          <t>每次撞击结算命中3种或以上不同标签的物品：+15分。</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2311,7 +2311,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>负价值物品完成结算后：额外+其负价值绝对值一半的分数，向下取整。每个物品每条链限1次。</t>
+          <t>负价值物品完成结算后：额外+其负价值绝对值一半的分数，向下取整。每个物品每次撞击结算限1次。</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>相邻两个同标签物品中，一个被撞时：另一个+2分，每条链每个物品限1次。</t>
+          <t>相邻两个同标签物品中，一个被撞时：另一个+2分，每次撞击结算每个物品限1次。</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2566,7 +2566,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>链结束时，若本局已经发生过污染结算、播种和大于等于5命中的撞击链：+45分，每局限1次。</t>
+          <t>本次撞击结算全部停止后时，若本局已经发生过污染结算、播种和大于等于5命中的撞击结算：+45分，每局限1次。</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -2724,7 +2724,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>黑墨水；消毒喷雾；腐蚀酸</t>
+          <t>黑墨滴；消毒喷雾；腐蚀酸</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -2882,7 +2882,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>鼓励用道具主动修正机械链。</t>
+          <t>鼓励用道具主动修正机械传动。</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>多目标道具；梦境钥匙；小水滴</t>
+          <t>多目标道具；梦值糖；小水滴</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -3155,12 +3155,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>每条撞击链第一次命中物品：+2分。</t>
+          <t>每次撞击结算第一次命中物品：+2分。</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>根源之梦；棒球；机械链</t>
+          <t>根源之梦；棒球；机械传动</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -3262,7 +3262,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>高San物品；特殊物品</t>
+          <t>高梦值消耗物品；特殊物品</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -3466,7 +3466,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>机械链；长条物品</t>
+          <t>机械传动；长条物品</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -3948,7 +3948,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>废弃物完成结算后：若其有污染，+其污染层数分。每个物品每条链限1次。</t>
+          <t>废弃物完成结算后：若其有污染，+其污染层数分。每个物品每次撞击结算限1次。</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -4101,7 +4101,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>污染层数大于等于3的物品完成结算后：+5分。每个物品每条链限1次。</t>
+          <t>污染层数大于等于3的物品完成结算后：+5分。每个物品每次撞击结算限1次。</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -4152,7 +4152,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>污染层数大于等于5的物品完成结算后：+污染层数x2分。每个物品每条链限1次。</t>
+          <t>污染层数大于等于5的物品完成结算后：+污染层数x2分。每个物品每次撞击结算限1次。</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -4310,7 +4310,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>黑墨水；消毒喷雾；腐蚀酸</t>
+          <t>黑墨滴；消毒喷雾；腐蚀酸</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -5172,12 +5172,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>机械/撞击链</t>
+          <t>机械/撞击结算</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>撞击链命中大于等于3个物品时：链结束+8分。</t>
+          <t>本次撞击结算命中大于等于3个物品时：在本次撞击结算全部停止后+8分。</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -5187,7 +5187,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>鼓励玩家做长链。</t>
+          <t>鼓励玩家做长路径。</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -5228,7 +5228,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>每条撞击链中，第一个被撞物品如果方向与撞击来源相同：+5分。</t>
+          <t>每次撞击结算中，第一个被撞物品如果方向与撞击来源相同：+5分。</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -5253,7 +5253,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>链长计数器</t>
+          <t>命中计数器</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -5274,12 +5274,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>机械/撞击链</t>
+          <t>机械/撞击结算</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>链结束：+本次命中物品数量分。若命中大于等于6，额外+8分。</t>
+          <t>本次撞击结算全部停止后：+本次命中物品数分。若命中大于等于6，额外+8分。</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -5289,7 +5289,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>把链长直接转化为收益。</t>
+          <t>把命中数直接转化为收益。</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -5330,7 +5330,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>每条撞击链第一次命中机械物品：+6分。</t>
+          <t>每次撞击结算第一次命中机械物品：+6分。</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -5381,17 +5381,17 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>机械物品成功传导撞击或曲线传动命中机械物品时：+2分，每条链最多触发5次。</t>
+          <t>机械物品成功传导撞击或曲线传动命中机械物品时：+2分，每次撞击结算最多触发5次。</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>机械长链；链长计数器；顺转弯管</t>
+          <t>机械长路径；命中计数器；左传动弯管</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>奖励机械链持续传导。</t>
+          <t>奖励机械传动持续传导。</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -5432,17 +5432,17 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>每个局内关卡第一次撞击链停止时，若最后被撞物品是机械：从该物品反方向发起一次机械撞击！</t>
+          <t>每个局内关卡第一次满足以下条件时触发：一次撞击结算全部停止后，最后被撞物品是机械。效果：从该物品反方向发起一次机械撞击！</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>机械链；终端压力表</t>
+          <t>机械传动；终端压力表</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>给机械链提供一次补偿性延伸。</t>
+          <t>给机械传动提供一次补偿性延伸。</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -5483,12 +5483,12 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>每条链第一次命中机械物品时：该物品本次触发双向传动！每条链限1次。</t>
+          <t>每次撞击结算第一次命中机械物品时：该物品本次触发双向传动！每次撞击结算限1次。</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>双轴转轮；曲线传动；长链</t>
+          <t>双轴转轮；曲线传动；长路径</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -5539,7 +5539,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>根源之梦；棒球；机械链</t>
+          <t>根源之梦；棒球；机械传动</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -5585,12 +5585,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>链结束：若本次链机械命中数大于等于8，+25分；若大于等于12，改为+45分。</t>
+          <t>本次撞击结算全部停止后：若本次命中机械物品数大于等于8，+25分；若大于等于12，改为+45分。</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>机械高阶长链；中央引擎；计数轮</t>
+          <t>机械高阶长路径；中央引擎；计数轮</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -5646,7 +5646,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>鼓励用道具主动修正机械链。</t>
+          <t>鼓励用道具主动修正机械传动。</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>每条撞击链命中3种或以上不同标签的物品：+15分。</t>
+          <t>每次撞击结算命中3种或以上不同标签的物品：+15分。</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -5817,7 +5817,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>负价值物品完成结算后：额外+其负价值绝对值一半的分数，向下取整。每个物品每条链限1次。</t>
+          <t>负价值物品完成结算后：额外+其负价值绝对值一半的分数，向下取整。每个物品每次撞击结算限1次。</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -5868,7 +5868,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>相邻两个同标签物品中，一个被撞时：另一个+2分，每条链每个物品限1次。</t>
+          <t>相邻两个同标签物品中，一个被撞时：另一个+2分，每次撞击结算每个物品限1次。</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -6072,7 +6072,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>链结束时，若本局已经发生过污染结算、播种和大于等于5命中的撞击链：+45分，每局限1次。</t>
+          <t>本次撞击结算全部停止后时，若本局已经发生过污染结算、播种和大于等于5命中的撞击结算：+45分，每局限1次。</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -6179,7 +6179,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>多目标道具；梦境钥匙；小水滴</t>
+          <t>多目标道具；梦值糖；小水滴</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">

</xml_diff>